<commit_message>
2025 SNA Update - Regional Accounts
</commit_message>
<xml_diff>
--- a/Data/National Accounts/PSA-02HFCE_2018PSNA_Ann.xlsx
+++ b/Data/National Accounts/PSA-02HFCE_2018PSNA_Ann.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Shared drives\QNAP\NAP Dissemination\As of January 2026\Tables\Prelim Q4 2025\NAP Q1 2000 to Q4 2025\Annl\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\Shared drives\QNAP\NAP Dissemination\As of April 2026\Tables\NAP Q1 2000 to Q4 2025\Annl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D655956B-79A0-4731-8DD4-63667CC83CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91DAAA7A-A6D4-4454-A50F-E3CA050AA2BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HFCE" sheetId="1" r:id="rId1"/>
@@ -217,9 +217,6 @@
     <t>2023 - 2024</t>
   </si>
   <si>
-    <t>As of January 2026</t>
-  </si>
-  <si>
     <t>Annual 2000 to 2025</t>
   </si>
   <si>
@@ -227,6 +224,9 @@
   </si>
   <si>
     <t>2024 - 2025</t>
+  </si>
+  <si>
+    <t>As of April 2026</t>
   </si>
 </sst>
 </file>
@@ -713,7 +713,7 @@
     </row>
     <row r="3" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:96" x14ac:dyDescent="0.2">
@@ -723,7 +723,7 @@
     </row>
     <row r="6" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:96" x14ac:dyDescent="0.2">
@@ -925,10 +925,10 @@
         <v>6853549.1516588246</v>
       </c>
       <c r="Z12" s="8">
-        <v>7253561.4106219551</v>
+        <v>7252163.3185486458</v>
       </c>
       <c r="AA12" s="8">
-        <v>7668107.3569288086</v>
+        <v>7659928.0205509737</v>
       </c>
       <c r="AB12" s="9"/>
       <c r="AC12" s="9"/>
@@ -1077,10 +1077,10 @@
         <v>354222.47225195228</v>
       </c>
       <c r="Z13" s="8">
-        <v>379665.70152991894</v>
+        <v>378021.32378579152</v>
       </c>
       <c r="AA13" s="8">
-        <v>382178.35208176239</v>
+        <v>382207.63664528128</v>
       </c>
       <c r="AB13" s="9"/>
       <c r="AC13" s="9"/>
@@ -1229,10 +1229,10 @@
         <v>264092.89607673243</v>
       </c>
       <c r="Z14" s="8">
-        <v>276462.78159096901</v>
+        <v>276504.00976352609</v>
       </c>
       <c r="AA14" s="8">
-        <v>283943.59826800274</v>
+        <v>284309.00662593008</v>
       </c>
       <c r="AB14" s="9"/>
       <c r="AC14" s="9"/>
@@ -1381,10 +1381,10 @@
         <v>2288370.7310069762</v>
       </c>
       <c r="Z15" s="8">
-        <v>2446525.1380855888</v>
+        <v>2446728.555972985</v>
       </c>
       <c r="AA15" s="8">
-        <v>2525525.9572911318</v>
+        <v>2526781.668296406</v>
       </c>
       <c r="AB15" s="9"/>
       <c r="AC15" s="9"/>
@@ -1533,10 +1533,10 @@
         <v>482907.40297373611</v>
       </c>
       <c r="Z16" s="8">
-        <v>512769.59179124155</v>
+        <v>512185.29672858666</v>
       </c>
       <c r="AA16" s="8">
-        <v>525420.75655138027</v>
+        <v>527731.90440869133</v>
       </c>
       <c r="AB16" s="9"/>
       <c r="AC16" s="9"/>
@@ -1685,10 +1685,10 @@
         <v>798192.55504901591</v>
       </c>
       <c r="Z17" s="8">
-        <v>902698.60629759915</v>
+        <v>903636.99943334237</v>
       </c>
       <c r="AA17" s="8">
-        <v>1012810.335900666</v>
+        <v>1012436.82298265</v>
       </c>
       <c r="AB17" s="9"/>
       <c r="AC17" s="9"/>
@@ -1837,10 +1837,10 @@
         <v>1803980.3159114744</v>
       </c>
       <c r="Z18" s="8">
-        <v>1980593.3007632052</v>
+        <v>1980516.5748665002</v>
       </c>
       <c r="AA18" s="8">
-        <v>2119622.0243572108</v>
+        <v>2117375.1722959727</v>
       </c>
       <c r="AB18" s="9"/>
       <c r="AC18" s="9"/>
@@ -1989,10 +1989,10 @@
         <v>496996.86583779933</v>
       </c>
       <c r="Z19" s="8">
-        <v>524252.61151829897</v>
+        <v>525174.99057351262</v>
       </c>
       <c r="AA19" s="8">
-        <v>549881.11482916865</v>
+        <v>550966.05744558736</v>
       </c>
       <c r="AB19" s="9"/>
       <c r="AC19" s="9"/>
@@ -2141,10 +2141,10 @@
         <v>286654.14915700798</v>
       </c>
       <c r="Z20" s="8">
-        <v>323464.92441998917</v>
+        <v>323012.62336940446</v>
       </c>
       <c r="AA20" s="8">
-        <v>350619.62855405954</v>
+        <v>350598.67263670306</v>
       </c>
       <c r="AB20" s="9"/>
       <c r="AC20" s="9"/>
@@ -2293,10 +2293,10 @@
         <v>916860.10352940368</v>
       </c>
       <c r="Z21" s="8">
-        <v>995314.90010947862</v>
+        <v>999583.03627352859</v>
       </c>
       <c r="AA21" s="8">
-        <v>1109890.3026707082</v>
+        <v>1110161.5656275761</v>
       </c>
       <c r="AB21" s="9"/>
       <c r="AC21" s="9"/>
@@ -2445,10 +2445,10 @@
         <v>1477881.4663575722</v>
       </c>
       <c r="Z22" s="8">
-        <v>1692667.6367904763</v>
+        <v>1694746.6595138737</v>
       </c>
       <c r="AA22" s="8">
-        <v>1843520.0444849543</v>
+        <v>1843383.7975543234</v>
       </c>
       <c r="AB22" s="9"/>
       <c r="AC22" s="9"/>
@@ -2597,10 +2597,10 @@
         <v>2580749.4352202103</v>
       </c>
       <c r="Z23" s="8">
-        <v>2849715.4939333918</v>
+        <v>2848630.1494251471</v>
       </c>
       <c r="AA23" s="8">
-        <v>3036761.8607270997</v>
+        <v>3036284.1094711591</v>
       </c>
       <c r="AB23" s="9"/>
       <c r="AC23" s="9"/>
@@ -2847,10 +2847,10 @@
         <v>18604457.545030702</v>
       </c>
       <c r="Z25" s="22">
-        <v>20137692.097452115</v>
+        <v>20140903.538254842</v>
       </c>
       <c r="AA25" s="22">
-        <v>21408281.332644954</v>
+        <v>21402164.434541255</v>
       </c>
       <c r="AB25" s="9"/>
       <c r="AC25" s="9"/>
@@ -3164,7 +3164,7 @@
     </row>
     <row r="32" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34" spans="1:96" x14ac:dyDescent="0.2">
@@ -3174,7 +3174,7 @@
     </row>
     <row r="35" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="36" spans="1:96" x14ac:dyDescent="0.2">
@@ -3376,10 +3376,10 @@
         <v>5485461.5751280217</v>
       </c>
       <c r="Z41" s="8">
-        <v>5562853.208788068</v>
+        <v>5561785.6176200565</v>
       </c>
       <c r="AA41" s="8">
-        <v>5813823.6885687625</v>
+        <v>5807656.0432445621</v>
       </c>
       <c r="AB41" s="9"/>
       <c r="AC41" s="9"/>
@@ -3528,10 +3528,10 @@
         <v>208586.20924864014</v>
       </c>
       <c r="Z42" s="8">
-        <v>213899.19798559108</v>
+        <v>213003.1812479455</v>
       </c>
       <c r="AA42" s="8">
-        <v>207829.66179079772</v>
+        <v>207849.44464062434</v>
       </c>
       <c r="AB42" s="9"/>
       <c r="AC42" s="9"/>
@@ -3680,10 +3680,10 @@
         <v>232443.53280160273</v>
       </c>
       <c r="Z43" s="8">
-        <v>236284.95390045649</v>
+        <v>236320.65637106469</v>
       </c>
       <c r="AA43" s="8">
-        <v>238168.82596829766</v>
+        <v>238478.61530469015</v>
       </c>
       <c r="AB43" s="9"/>
       <c r="AC43" s="9"/>
@@ -3832,10 +3832,10 @@
         <v>1937670.7077466038</v>
       </c>
       <c r="Z44" s="8">
-        <v>2038772.0417034051</v>
+        <v>2038938.0202471504</v>
       </c>
       <c r="AA44" s="8">
-        <v>2055896.4336929899</v>
+        <v>2056893.7280070833</v>
       </c>
       <c r="AB44" s="9"/>
       <c r="AC44" s="9"/>
@@ -3984,10 +3984,10 @@
         <v>408076.47724212188</v>
       </c>
       <c r="Z45" s="8">
-        <v>421120.50234056893</v>
+        <v>420637.98087730224</v>
       </c>
       <c r="AA45" s="8">
-        <v>422201.33915592264</v>
+        <v>424061.6353368368</v>
       </c>
       <c r="AB45" s="9"/>
       <c r="AC45" s="9"/>
@@ -4136,10 +4136,10 @@
         <v>686248.25037239364</v>
       </c>
       <c r="Z46" s="8">
-        <v>754723.16311876278</v>
+        <v>755477.70263676043</v>
       </c>
       <c r="AA46" s="8">
-        <v>825473.56679974869</v>
+        <v>825171.75887761731</v>
       </c>
       <c r="AB46" s="9"/>
       <c r="AC46" s="9"/>
@@ -4288,10 +4288,10 @@
         <v>1372864.2504209473</v>
       </c>
       <c r="Z47" s="8">
-        <v>1496402.0513733246</v>
+        <v>1496340.998535573</v>
       </c>
       <c r="AA47" s="8">
-        <v>1608449.5876347541</v>
+        <v>1606892.3028661709</v>
       </c>
       <c r="AB47" s="9"/>
       <c r="AC47" s="9"/>
@@ -4440,10 +4440,10 @@
         <v>487836.33144416905</v>
       </c>
       <c r="Z48" s="8">
-        <v>512532.57860805659</v>
+        <v>513449.36603211914</v>
       </c>
       <c r="AA48" s="8">
-        <v>534981.27305097762</v>
+        <v>536076.30021088314</v>
       </c>
       <c r="AB48" s="9"/>
       <c r="AC48" s="9"/>
@@ -4592,10 +4592,10 @@
         <v>261856.2734591449</v>
       </c>
       <c r="Z49" s="8">
-        <v>286249.69045336795</v>
+        <v>285857.19194377854</v>
       </c>
       <c r="AA49" s="8">
-        <v>303720.63039504387</v>
+        <v>303691.34749998274</v>
       </c>
       <c r="AB49" s="9"/>
       <c r="AC49" s="9"/>
@@ -4744,10 +4744,10 @@
         <v>839365.86430522939</v>
       </c>
       <c r="Z50" s="8">
-        <v>873586.32457309763</v>
+        <v>877365.77996879071</v>
       </c>
       <c r="AA50" s="8">
-        <v>938705.76435978687</v>
+        <v>938945.44470473495</v>
       </c>
       <c r="AB50" s="9"/>
       <c r="AC50" s="9"/>
@@ -4896,10 +4896,10 @@
         <v>1211225.7496792087</v>
       </c>
       <c r="Z51" s="8">
-        <v>1324816.1353516914</v>
+        <v>1326444.1879137582</v>
       </c>
       <c r="AA51" s="8">
-        <v>1411251.6388390658</v>
+        <v>1411150.5323371522</v>
       </c>
       <c r="AB51" s="9"/>
       <c r="AC51" s="9"/>
@@ -5048,10 +5048,10 @@
         <v>2245566.0873440439</v>
       </c>
       <c r="Z52" s="8">
-        <v>2402886.2157230945</v>
+        <v>2401991.0343113309</v>
       </c>
       <c r="AA52" s="8">
-        <v>2499080.467035152</v>
+        <v>2498793.9162581377</v>
       </c>
       <c r="AB52" s="9"/>
       <c r="AC52" s="9"/>
@@ -5298,10 +5298,10 @@
         <v>15377201.309192125</v>
       </c>
       <c r="Z54" s="22">
-        <v>16124126.063919485</v>
+        <v>16127611.71770563</v>
       </c>
       <c r="AA54" s="22">
-        <v>16859582.877291299</v>
+        <v>16855661.069288477</v>
       </c>
       <c r="AB54" s="9"/>
       <c r="AC54" s="9"/>
@@ -5615,7 +5615,7 @@
     </row>
     <row r="61" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="63" spans="1:96" x14ac:dyDescent="0.2">
@@ -5625,7 +5625,7 @@
     </row>
     <row r="64" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="65" spans="1:91" x14ac:dyDescent="0.2">
@@ -5741,7 +5741,7 @@
         <v>56</v>
       </c>
       <c r="Z68" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AA68" s="20"/>
     </row>
@@ -5822,10 +5822,10 @@
         <v>8.2287463002206351</v>
       </c>
       <c r="Y70" s="18">
-        <v>5.8365709519470244</v>
+        <v>5.8161714181817814</v>
       </c>
       <c r="Z70" s="26">
-        <v>5.7150677141824673</v>
+        <v>5.622662977809668</v>
       </c>
       <c r="AA70" s="26"/>
       <c r="AB70" s="9"/>
@@ -5967,10 +5967,10 @@
         <v>7.8718776551386185</v>
       </c>
       <c r="Y71" s="18">
-        <v>7.1828388290027192</v>
+        <v>6.7186170833655012</v>
       </c>
       <c r="Z71" s="26">
-        <v>0.66180604192540216</v>
+        <v>1.1074277021107832</v>
       </c>
       <c r="AA71" s="26"/>
       <c r="AB71" s="9"/>
@@ -6112,10 +6112,10 @@
         <v>-5.679722243469854</v>
       </c>
       <c r="Y72" s="18">
-        <v>4.6839145232602277</v>
+        <v>4.6995257620211106</v>
       </c>
       <c r="Z72" s="26">
-        <v>2.7059037147726173</v>
+        <v>2.8227427403599137</v>
       </c>
       <c r="AA72" s="26"/>
       <c r="AB72" s="9"/>
@@ -6257,10 +6257,10 @@
         <v>9.7128003788330801</v>
       </c>
       <c r="Y73" s="18">
-        <v>6.9112231220077831</v>
+        <v>6.9201123235973654</v>
       </c>
       <c r="Z73" s="26">
-        <v>3.229103105286768</v>
+        <v>3.2718428093706677</v>
       </c>
       <c r="AA73" s="26"/>
       <c r="AB73" s="9"/>
@@ -6402,10 +6402,10 @@
         <v>3.9551394054073938</v>
       </c>
       <c r="Y74" s="18">
-        <v>6.18383330502175</v>
+        <v>6.0628380460845648</v>
       </c>
       <c r="Z74" s="26">
-        <v>2.4672221135314913</v>
+        <v>3.0353482966815903</v>
       </c>
       <c r="AA74" s="26"/>
       <c r="AB74" s="9"/>
@@ -6547,10 +6547,10 @@
         <v>11.275348003970961</v>
       </c>
       <c r="Y75" s="18">
-        <v>13.092837134037879</v>
+        <v>13.210401890788276</v>
       </c>
       <c r="Z75" s="26">
-        <v>12.198061327987205</v>
+        <v>12.04021345048227</v>
       </c>
       <c r="AA75" s="26"/>
       <c r="AB75" s="9"/>
@@ -6692,10 +6692,10 @@
         <v>18.838729016332564</v>
       </c>
       <c r="Y76" s="18">
-        <v>9.7901835898079383</v>
+        <v>9.7859304449134044</v>
       </c>
       <c r="Z76" s="26">
-        <v>7.0195493209248099</v>
+        <v>6.9102475165448993</v>
       </c>
       <c r="AA76" s="26"/>
       <c r="AB76" s="9"/>
@@ -6837,10 +6837,10 @@
         <v>5.3149886319968829</v>
       </c>
       <c r="Y77" s="18">
-        <v>5.4840880403851173</v>
+        <v>5.6696785578743487</v>
       </c>
       <c r="Z77" s="26">
-        <v>4.8885790452519444</v>
+        <v>4.910947271862625</v>
       </c>
       <c r="AA77" s="26"/>
       <c r="AB77" s="9"/>
@@ -6982,10 +6982,10 @@
         <v>21.412244450861209</v>
       </c>
       <c r="Y78" s="18">
-        <v>12.841528849742545</v>
+        <v>12.683742523636738</v>
       </c>
       <c r="Z78" s="26">
-        <v>8.3949455053780468</v>
+        <v>8.540238762046954</v>
       </c>
       <c r="AA78" s="26"/>
       <c r="AB78" s="9"/>
@@ -7127,10 +7127,10 @@
         <v>10.27076882017117</v>
       </c>
       <c r="Y79" s="18">
-        <v>8.556899387165771</v>
+        <v>9.0224160071626471</v>
       </c>
       <c r="Z79" s="26">
-        <v>11.51147265540051</v>
+        <v>11.062465582277909</v>
       </c>
       <c r="AA79" s="26"/>
       <c r="AB79" s="9"/>
@@ -7272,10 +7272,10 @@
         <v>27.040020803690723</v>
       </c>
       <c r="Y80" s="18">
-        <v>14.533382772724806</v>
+        <v>14.674058650372928</v>
       </c>
       <c r="Z80" s="26">
-        <v>8.9121103526569811</v>
+        <v>8.7704635501736306</v>
       </c>
       <c r="AA80" s="26"/>
       <c r="AB80" s="9"/>
@@ -7417,10 +7417,10 @@
         <v>12.412994588465239</v>
       </c>
       <c r="Y81" s="18">
-        <v>10.422013661711077</v>
+        <v>10.379958261313305</v>
       </c>
       <c r="Z81" s="26">
-        <v>6.5636856448266769</v>
+        <v>6.5875157602990555</v>
       </c>
       <c r="AA81" s="26"/>
       <c r="AB81" s="9"/>
@@ -7655,10 +7655,10 @@
         <v>11.237116864864774</v>
       </c>
       <c r="Y83" s="18">
-        <v>8.2412214852829493</v>
+        <v>8.2584831592390486</v>
       </c>
       <c r="Z83" s="26">
-        <v>6.3095077084508517</v>
+        <v>6.2621862712902754</v>
       </c>
       <c r="AA83" s="26"/>
       <c r="AB83" s="9"/>
@@ -7958,7 +7958,7 @@
     </row>
     <row r="90" spans="1:91" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="92" spans="1:91" x14ac:dyDescent="0.2">
@@ -7968,7 +7968,7 @@
     </row>
     <row r="93" spans="1:91" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="94" spans="1:91" x14ac:dyDescent="0.2">
@@ -8084,7 +8084,7 @@
         <v>56</v>
       </c>
       <c r="Z97" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AA97" s="20"/>
     </row>
@@ -8165,10 +8165,10 @@
         <v>0.54997122189965353</v>
       </c>
       <c r="Y99" s="18">
-        <v>1.4108499822686298</v>
+        <v>1.391387788369542</v>
       </c>
       <c r="Z99" s="26">
-        <v>4.5115423751289683</v>
+        <v>4.4207102274056496</v>
       </c>
       <c r="AA99" s="21"/>
       <c r="AB99" s="9"/>
@@ -8310,10 +8310,10 @@
         <v>-1.5183005851512661</v>
       </c>
       <c r="Y100" s="18">
-        <v>2.5471428605415127</v>
+        <v>2.1175762363273947</v>
       </c>
       <c r="Z100" s="26">
-        <v>-2.8375684677425568</v>
+        <v>-2.4195585141622615</v>
       </c>
       <c r="AA100" s="21"/>
       <c r="AB100" s="9"/>
@@ -8455,10 +8455,10 @@
         <v>-9.5812430491842804</v>
       </c>
       <c r="Y101" s="18">
-        <v>1.6526255011502116</v>
+        <v>1.6679851328757849</v>
       </c>
       <c r="Z101" s="26">
-        <v>0.79728820508597664</v>
+        <v>0.9131486712854695</v>
       </c>
       <c r="AA101" s="21"/>
       <c r="AB101" s="9"/>
@@ -8600,10 +8600,10 @@
         <v>4.671770980355717</v>
       </c>
       <c r="Y102" s="18">
-        <v>5.2176736507709478</v>
+        <v>5.2262395305709362</v>
       </c>
       <c r="Z102" s="26">
-        <v>0.8399365715883107</v>
+        <v>0.88064019512256664</v>
       </c>
       <c r="AA102" s="21"/>
       <c r="AB102" s="9"/>
@@ -8745,10 +8745,10 @@
         <v>-1.0540353294230584</v>
       </c>
       <c r="Y103" s="18">
-        <v>3.1964658160650998</v>
+        <v>3.0782229154873164</v>
       </c>
       <c r="Z103" s="26">
-        <v>0.25665737225959617</v>
+        <v>0.81391947831102129</v>
       </c>
       <c r="AA103" s="21"/>
       <c r="AB103" s="9"/>
@@ -8890,10 +8890,10 @@
         <v>7.1424192160312003</v>
       </c>
       <c r="Y104" s="18">
-        <v>9.9781548017370056</v>
+        <v>10.088106195797124</v>
       </c>
       <c r="Z104" s="26">
-        <v>9.3743517011750441</v>
+        <v>9.2251638926749848</v>
       </c>
       <c r="AA104" s="21"/>
       <c r="AB104" s="9"/>
@@ -9035,10 +9035,10 @@
         <v>16.941603874678762</v>
       </c>
       <c r="Y105" s="18">
-        <v>8.9985445330445657</v>
+        <v>8.9940974190831469</v>
       </c>
       <c r="Z105" s="26">
-        <v>7.4877962215166463</v>
+        <v>7.3881090231966624</v>
       </c>
       <c r="AA105" s="21"/>
       <c r="AB105" s="9"/>
@@ -9180,10 +9180,10 @@
         <v>4.6135857156055664</v>
       </c>
       <c r="Y106" s="18">
-        <v>5.0624042475020019</v>
+        <v>5.2503335518546521</v>
       </c>
       <c r="Z106" s="26">
-        <v>4.3799546370081544</v>
+        <v>4.4068482065958108</v>
       </c>
       <c r="AA106" s="21"/>
       <c r="AB106" s="9"/>
@@ -9325,10 +9325,10 @@
         <v>16.549877188370374</v>
       </c>
       <c r="Y107" s="18">
-        <v>9.3155747891711087</v>
+        <v>9.165683971431875</v>
       </c>
       <c r="Z107" s="26">
-        <v>6.1033917325832334</v>
+        <v>6.2388339558417556</v>
       </c>
       <c r="AA107" s="21"/>
       <c r="AB107" s="9"/>
@@ -9470,10 +9470,10 @@
         <v>6.4900029957358072</v>
       </c>
       <c r="Y108" s="18">
-        <v>4.0769420967808401</v>
+        <v>4.5272171861569603</v>
       </c>
       <c r="Z108" s="26">
-        <v>7.4542650170847935</v>
+        <v>7.0186991722123793</v>
       </c>
       <c r="AA108" s="21"/>
       <c r="AB108" s="9"/>
@@ -9615,10 +9615,10 @@
         <v>19.029574531214323</v>
       </c>
       <c r="Y109" s="18">
-        <v>9.3781349762888482</v>
+        <v>9.5125486116081106</v>
       </c>
       <c r="Z109" s="26">
-        <v>6.5243395804829021</v>
+        <v>6.3859712451694435</v>
       </c>
       <c r="AA109" s="21"/>
       <c r="AB109" s="9"/>
@@ -9760,10 +9760,10 @@
         <v>8.4218854324208223</v>
       </c>
       <c r="Y110" s="18">
-        <v>7.0058115530735421</v>
+        <v>6.965947154657087</v>
       </c>
       <c r="Z110" s="26">
-        <v>4.0032795012355535</v>
+        <v>4.0301100447096729</v>
       </c>
       <c r="AA110" s="21"/>
       <c r="AB110" s="9"/>
@@ -9998,10 +9998,10 @@
         <v>5.5376377823433955</v>
       </c>
       <c r="Y112" s="18">
-        <v>4.8573517359161258</v>
+        <v>4.8800194094157376</v>
       </c>
       <c r="Z112" s="26">
-        <v>4.5612196931251106</v>
+        <v>4.5143035703393224</v>
       </c>
       <c r="AA112" s="21"/>
       <c r="AB112" s="9"/>
@@ -10298,7 +10298,7 @@
     </row>
     <row r="118" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="120" spans="1:96" x14ac:dyDescent="0.2">
@@ -10308,7 +10308,7 @@
     </row>
     <row r="121" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="122" spans="1:96" x14ac:dyDescent="0.2">
@@ -10510,10 +10510,10 @@
         <v>124.94024537030639</v>
       </c>
       <c r="Z127" s="26">
-        <v>130.39282430035982</v>
+        <v>130.39271588558495</v>
       </c>
       <c r="AA127" s="26">
-        <v>131.89439115613308</v>
+        <v>131.89362392528335</v>
       </c>
       <c r="AB127" s="9"/>
       <c r="AC127" s="9"/>
@@ -10662,10 +10662,10 @@
         <v>169.82065762061478</v>
       </c>
       <c r="Z128" s="26">
-        <v>177.49748718342292</v>
+        <v>177.47214927544078</v>
       </c>
       <c r="AA128" s="26">
-        <v>183.8901862172421</v>
+        <v>183.88677309488395</v>
       </c>
       <c r="AB128" s="9"/>
       <c r="AC128" s="9"/>
@@ -10814,10 +10814,10 @@
         <v>113.61593626360143</v>
       </c>
       <c r="Z129" s="26">
-        <v>117.00397212233788</v>
+        <v>117.00374144584573</v>
       </c>
       <c r="AA129" s="26">
-        <v>119.21946422400305</v>
+        <v>119.21782012306853</v>
       </c>
       <c r="AB129" s="9"/>
       <c r="AC129" s="9"/>
@@ -10966,10 +10966,10 @@
         <v>118.09905170462198</v>
       </c>
       <c r="Z130" s="26">
-        <v>119.99993564957383</v>
+        <v>120.00014378447874</v>
       </c>
       <c r="AA130" s="26">
-        <v>122.84305356542451</v>
+        <v>122.84454145059772</v>
       </c>
       <c r="AB130" s="9"/>
       <c r="AC130" s="9"/>
@@ -11118,10 +11118,10 @@
         <v>118.33747591562724</v>
       </c>
       <c r="Z131" s="26">
-        <v>121.7631506757071</v>
+        <v>121.76392052385498</v>
       </c>
       <c r="AA131" s="26">
-        <v>124.44791331117446</v>
+        <v>124.44698138974731</v>
       </c>
       <c r="AB131" s="9"/>
       <c r="AC131" s="9"/>
@@ -11270,10 +11270,10 @@
         <v>116.31250857337349</v>
       </c>
       <c r="Z132" s="26">
-        <v>119.60658562105786</v>
+        <v>119.61133945839539</v>
       </c>
       <c r="AA132" s="26">
-        <v>122.69446008152593</v>
+        <v>122.69407091194529</v>
       </c>
       <c r="AB132" s="9"/>
       <c r="AC132" s="9"/>
@@ -11422,10 +11422,10 @@
         <v>131.40267257730241</v>
       </c>
       <c r="Z133" s="26">
-        <v>132.35702924528294</v>
+        <v>132.35730203240948</v>
       </c>
       <c r="AA133" s="26">
-        <v>131.78044501066037</v>
+        <v>131.76833123907977</v>
       </c>
       <c r="AB133" s="9"/>
       <c r="AC133" s="9"/>
@@ -11574,10 +11574,10 @@
         <v>101.87778847190651</v>
       </c>
       <c r="Z134" s="26">
-        <v>102.28669032943658</v>
+        <v>102.28369637146655</v>
       </c>
       <c r="AA134" s="26">
-        <v>102.78511464396087</v>
+        <v>102.77754439598372</v>
       </c>
       <c r="AB134" s="9"/>
       <c r="AC134" s="9"/>
@@ -11726,10 +11726,10 @@
         <v>109.47003307206695</v>
       </c>
       <c r="Z135" s="26">
-        <v>113.0009691565706</v>
+        <v>112.99789981597999</v>
       </c>
       <c r="AA135" s="26">
-        <v>115.44149243270535</v>
+        <v>115.44572327228487</v>
       </c>
       <c r="AB135" s="9"/>
       <c r="AC135" s="9"/>
@@ -11878,10 +11878,10 @@
         <v>109.23247448099629</v>
       </c>
       <c r="Z136" s="26">
-        <v>113.93434994485143</v>
+        <v>113.93002315511842</v>
       </c>
       <c r="AA136" s="26">
-        <v>118.23622958442917</v>
+        <v>118.23493813069005</v>
       </c>
       <c r="AB136" s="9"/>
       <c r="AC136" s="9"/>
@@ -12030,10 +12030,10 @@
         <v>122.01536061704326</v>
       </c>
       <c r="Z137" s="26">
-        <v>127.76623046949329</v>
+        <v>127.76614914943269</v>
       </c>
       <c r="AA137" s="26">
-        <v>130.63014374966355</v>
+        <v>130.62984814960211</v>
       </c>
       <c r="AB137" s="9"/>
       <c r="AC137" s="9"/>
@@ -12182,10 +12182,10 @@
         <v>114.92645216568116</v>
       </c>
       <c r="Z138" s="26">
-        <v>118.59552380327065</v>
+        <v>118.59453714580042</v>
       </c>
       <c r="AA138" s="26">
-        <v>121.51516931064808</v>
+        <v>121.50998486573457</v>
       </c>
       <c r="AB138" s="9"/>
       <c r="AC138" s="9"/>
@@ -12432,10 +12432,10 @@
         <v>120.98727961576077</v>
       </c>
       <c r="Z140" s="26">
-        <v>124.89168105993464</v>
+        <v>124.88460096136392</v>
       </c>
       <c r="AA140" s="26">
-        <v>126.97989913783951</v>
+        <v>126.97315368743764</v>
       </c>
       <c r="AB140" s="9"/>
       <c r="AC140" s="9"/>
@@ -12553,7 +12553,7 @@
     </row>
     <row r="147" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="149" spans="1:96" x14ac:dyDescent="0.2">
@@ -12563,7 +12563,7 @@
     </row>
     <row r="150" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="151" spans="1:96" x14ac:dyDescent="0.2">
@@ -12765,10 +12765,10 @@
         <v>36.838210063745855</v>
       </c>
       <c r="Z156" s="26">
-        <v>36.019824791837486</v>
+        <v>36.007139921871783</v>
       </c>
       <c r="AA156" s="26">
-        <v>35.818416423909298</v>
+        <v>35.79043626161711</v>
       </c>
       <c r="AB156" s="9"/>
       <c r="AC156" s="9"/>
@@ -12917,10 +12917,10 @@
         <v>1.903965602837832</v>
       </c>
       <c r="Z157" s="26">
-        <v>1.8853486273035003</v>
+        <v>1.8768836416290493</v>
       </c>
       <c r="AA157" s="26">
-        <v>1.7851893206344789</v>
+        <v>1.7858363709627001</v>
       </c>
       <c r="AB157" s="9"/>
       <c r="AC157" s="9"/>
@@ -13069,10 +13069,10 @@
         <v>1.4195140892311171</v>
       </c>
       <c r="Z158" s="26">
-        <v>1.3728622935194641</v>
+        <v>1.3728480911412202</v>
       </c>
       <c r="AA158" s="26">
-        <v>1.3263259850524489</v>
+        <v>1.3284124019114616</v>
       </c>
       <c r="AB158" s="9"/>
       <c r="AC158" s="9"/>
@@ -13221,10 +13221,10 @@
         <v>12.300120685960048</v>
       </c>
       <c r="Z159" s="26">
-        <v>12.148984730952019</v>
+        <v>12.148057565172113</v>
       </c>
       <c r="AA159" s="26">
-        <v>11.79695799979992</v>
+        <v>11.806196873333043</v>
       </c>
       <c r="AB159" s="9"/>
       <c r="AC159" s="9"/>
@@ -13373,10 +13373,10 @@
         <v>2.5956543038403281</v>
       </c>
       <c r="Z160" s="26">
-        <v>2.5463175686161117</v>
+        <v>2.5430105246061179</v>
       </c>
       <c r="AA160" s="26">
-        <v>2.4542874245125845</v>
+        <v>2.4657875422963174</v>
       </c>
       <c r="AB160" s="9"/>
       <c r="AC160" s="9"/>
@@ -13525,10 +13525,10 @@
         <v>4.2903296326541653</v>
       </c>
       <c r="Z161" s="26">
-        <v>4.4826318821897742</v>
+        <v>4.4865762735867811</v>
       </c>
       <c r="AA161" s="26">
-        <v>4.7309278132301857</v>
+        <v>4.7305347367047794</v>
       </c>
       <c r="AB161" s="9"/>
       <c r="AC161" s="9"/>
@@ -13677,10 +13677,10 @@
         <v>9.696495109008552</v>
       </c>
       <c r="Z162" s="26">
-        <v>9.8352546616491168</v>
+        <v>9.8333054974658154</v>
       </c>
       <c r="AA162" s="26">
-        <v>9.9009443655107994</v>
+        <v>9.8932758823154874</v>
       </c>
       <c r="AB162" s="9"/>
       <c r="AC162" s="9"/>
@@ -13829,10 +13829,10 @@
         <v>2.6713859548705221</v>
       </c>
       <c r="Z163" s="26">
-        <v>2.6033400897247261</v>
+        <v>2.6075046215082449</v>
       </c>
       <c r="AA163" s="26">
-        <v>2.5685439493485571</v>
+        <v>2.5743473709433586</v>
       </c>
       <c r="AB163" s="9"/>
       <c r="AC163" s="9"/>
@@ -13981,10 +13981,10 @@
         <v>1.540782086568141</v>
       </c>
       <c r="Z164" s="26">
-        <v>1.6062661145808015</v>
+        <v>1.603764313531848</v>
       </c>
       <c r="AA164" s="26">
-        <v>1.6377756957977212</v>
+        <v>1.6381458693536011</v>
       </c>
       <c r="AB164" s="9"/>
       <c r="AC164" s="9"/>
@@ -14133,10 +14133,10 @@
         <v>4.9281743437571999</v>
       </c>
       <c r="Z165" s="26">
-        <v>4.9425470172692183</v>
+        <v>4.9629503183656078</v>
       </c>
       <c r="AA165" s="26">
-        <v>5.1843970350775619</v>
+        <v>5.1871462301068521</v>
       </c>
       <c r="AB165" s="9"/>
       <c r="AC165" s="9"/>
@@ -14285,10 +14285,10 @@
         <v>7.9436955513509089</v>
       </c>
       <c r="Z166" s="26">
-        <v>8.4054698452988958</v>
+        <v>8.4144519946433309</v>
       </c>
       <c r="AA166" s="26">
-        <v>8.61124728248884</v>
+        <v>8.6130718376280679</v>
       </c>
       <c r="AB166" s="9"/>
       <c r="AC166" s="9"/>
@@ -14437,10 +14437,10 @@
         <v>13.871672576175353</v>
       </c>
       <c r="Z167" s="26">
-        <v>14.151152377058873</v>
+        <v>14.143507236478097</v>
       </c>
       <c r="AA167" s="26">
-        <v>14.184986704637598</v>
+        <v>14.186808622827218</v>
       </c>
       <c r="AB167" s="9"/>
       <c r="AC167" s="9"/>
@@ -15004,7 +15004,7 @@
     </row>
     <row r="176" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A176" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="178" spans="1:96" x14ac:dyDescent="0.2">
@@ -15014,7 +15014,7 @@
     </row>
     <row r="179" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="180" spans="1:96" x14ac:dyDescent="0.2">
@@ -15216,10 +15216,10 @@
         <v>35.672691439949759</v>
       </c>
       <c r="Z185" s="26">
-        <v>34.50018429982331</v>
+        <v>34.486108141567385</v>
       </c>
       <c r="AA185" s="26">
-        <v>34.483793169044432</v>
+        <v>34.45522557300518</v>
       </c>
       <c r="AB185" s="9"/>
       <c r="AC185" s="9"/>
@@ -15368,10 +15368,10 @@
         <v>1.356464060361571</v>
       </c>
       <c r="Z186" s="26">
-        <v>1.326578551529856</v>
+        <v>1.3207360455863459</v>
       </c>
       <c r="AA186" s="26">
-        <v>1.2327093932479789</v>
+        <v>1.2331135740462431</v>
       </c>
       <c r="AB186" s="9"/>
       <c r="AC186" s="9"/>
@@ -15520,10 +15520,10 @@
         <v>1.5116114312859619</v>
       </c>
       <c r="Z187" s="26">
-        <v>1.4654124692635893</v>
+        <v>1.4653171251117179</v>
       </c>
       <c r="AA187" s="26">
-        <v>1.4126614383152665</v>
+        <v>1.4148280172719263</v>
       </c>
       <c r="AB187" s="9"/>
       <c r="AC187" s="9"/>
@@ -15672,10 +15672,10 @@
         <v>12.600932177354734</v>
       </c>
       <c r="Z188" s="26">
-        <v>12.644232832348724</v>
+        <v>12.642529197356053</v>
       </c>
       <c r="AA188" s="26">
-        <v>12.194230715293326</v>
+        <v>12.202984620726658</v>
       </c>
       <c r="AB188" s="9"/>
       <c r="AC188" s="9"/>
@@ -15824,10 +15824,10 @@
         <v>2.6537759962743253</v>
       </c>
       <c r="Z189" s="26">
-        <v>2.6117415646042286</v>
+        <v>2.6081851934437794</v>
       </c>
       <c r="AA189" s="26">
-        <v>2.5042217368532818</v>
+        <v>2.5158410197834953</v>
       </c>
       <c r="AB189" s="9"/>
       <c r="AC189" s="9"/>
@@ -15976,10 +15976,10 @@
         <v>4.4627643000431476</v>
       </c>
       <c r="Z190" s="26">
-        <v>4.6807074078116155</v>
+        <v>4.6843743256006247</v>
       </c>
       <c r="AA190" s="26">
-        <v>4.896168385705467</v>
+        <v>4.8955170342212515</v>
       </c>
       <c r="AB190" s="9"/>
       <c r="AC190" s="9"/>
@@ -16128,10 +16128,10 @@
         <v>8.9279201254930687</v>
       </c>
       <c r="Z191" s="26">
-        <v>9.2805157032465928</v>
+        <v>9.2781313484427539</v>
       </c>
       <c r="AA191" s="26">
-        <v>9.5402691711977372</v>
+        <v>9.5332499642744768</v>
       </c>
       <c r="AB191" s="9"/>
       <c r="AC191" s="9"/>
@@ -16280,10 +16280,10 @@
         <v>3.1724650125543463</v>
       </c>
       <c r="Z192" s="26">
-        <v>3.1786688877044735</v>
+        <v>3.1836664660548033</v>
       </c>
       <c r="AA192" s="26">
-        <v>3.1731584164609474</v>
+        <v>3.1803932103715016</v>
       </c>
       <c r="AB192" s="9"/>
       <c r="AC192" s="9"/>
@@ -16432,10 +16432,10 @@
         <v>1.7028864238293706</v>
       </c>
       <c r="Z193" s="26">
-        <v>1.7752880951104757</v>
+        <v>1.7724706977534155</v>
       </c>
       <c r="AA193" s="26">
-        <v>1.801471795628673</v>
+        <v>1.8017172168543274</v>
       </c>
       <c r="AB193" s="9"/>
       <c r="AC193" s="9"/>
@@ -16584,10 +16584,10 @@
         <v>5.4585086546501573</v>
       </c>
       <c r="Z194" s="26">
-        <v>5.4178832459509101</v>
+        <v>5.4401469686027877</v>
       </c>
       <c r="AA194" s="26">
-        <v>5.567787597071332</v>
+        <v>5.5705050122034185</v>
       </c>
       <c r="AB194" s="9"/>
       <c r="AC194" s="9"/>
@@ -16736,10 +16736,10 @@
         <v>7.8767633025339068</v>
       </c>
       <c r="Z195" s="26">
-        <v>8.2163593245291988</v>
+        <v>8.2246783412917068</v>
       </c>
       <c r="AA195" s="26">
-        <v>8.3706201340243407</v>
+        <v>8.3719678898166201</v>
       </c>
       <c r="AB195" s="9"/>
       <c r="AC195" s="9"/>
@@ -16888,10 +16888,10 @@
         <v>14.603217075669667</v>
       </c>
       <c r="Z196" s="26">
-        <v>14.902427618077033</v>
+        <v>14.893656149188633</v>
       </c>
       <c r="AA196" s="26">
-        <v>14.822908047157215</v>
+        <v>14.824656867424887</v>
       </c>
       <c r="AB196" s="9"/>
       <c r="AC196" s="9"/>

</xml_diff>